<commit_message>
[S3] feat: Sprint 3 integration tests and retrospective
</commit_message>
<xml_diff>
--- a/reports/screener_output.xlsx
+++ b/reports/screener_output.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Compounder" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value Pick" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dividend Aristocrat" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Growth Rocket" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Light Champion" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Health" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Quality Compounder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Value Pick" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dividend Aristocrat" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Growth Rocket" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Asset Light Champion" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Financial Health" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +23,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,57 +423,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>in_quality_compounder</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>in_value_pick</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>in_dividend_aristocrat</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>in_growth_rocket</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>in_asset_light_champion</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>in_financial_health</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>total_presets_matched</t>
         </is>
@@ -4272,47 +4260,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>return_on_equity_pct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>debt_to_equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>revenue_cagr_3yr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>operating_profit_margin_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
@@ -5278,42 +5266,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>pe_ratio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>pb_ratio</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>return_on_equity_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>debt_to_equity</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
@@ -5398,42 +5386,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>dividend_payout_ratio_pct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>debt_to_equity</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>return_on_equity_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
@@ -6222,37 +6210,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>revenue_cagr_3yr</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>pat_cagr_3yr</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>operating_profit_margin_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
@@ -6592,37 +6580,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>capex_intensity_pct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>return_on_equity_pct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>operating_profit_margin_pct</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>
@@ -6730,42 +6718,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>company_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>broad_sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>interest_coverage</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>debt_to_equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>cfo_quality_score</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>free_cash_flow_cr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>composite_ranking_score</t>
         </is>

</xml_diff>